<commit_message>
Oculta subtopicos de Engenharia ate expansao no menu lateral e atualiza planilha
</commit_message>
<xml_diff>
--- a/BALANÇA_ATERRO.xlsx
+++ b/BALANÇA_ATERRO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muril\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B28A8D-314D-4EF4-B791-447C2C3D1198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44FACFD-D991-4826-B4E5-5AC19106AD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DDC835EE-E68E-4405-84CA-BBF9A30D9944}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DDC835EE-E68E-4405-84CA-BBF9A30D9944}"/>
   </bookViews>
   <sheets>
     <sheet name="AGOSTO" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="62">
   <si>
     <t>Entulho</t>
   </si>
@@ -283,7 +283,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -365,6 +365,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF7D7D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -886,7 +892,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1110,6 +1116,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5234,14 +5243,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>277468</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>252621</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>382243</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>357396</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
@@ -5258,7 +5267,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5106643" y="2133600"/>
+          <a:off x="3872121" y="2133600"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5301,14 +5310,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>258418</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>233571</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>363193</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>338346</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -5325,7 +5334,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5087593" y="1381125"/>
+          <a:off x="3853071" y="1381125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5368,14 +5377,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>263180</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238333</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>367955</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>343108</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -5392,7 +5401,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5092355" y="619125"/>
+          <a:off x="3857833" y="619125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5435,14 +5444,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>272705</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>247858</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>377480</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352633</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -5459,7 +5468,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5101880" y="1952625"/>
+          <a:off x="3867358" y="1952625"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5502,14 +5511,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>263180</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238333</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>367955</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>343108</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -5526,7 +5535,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5092355" y="1000125"/>
+          <a:off x="3857833" y="1000125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5569,23 +5578,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>276069</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>45243</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>232838</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>380844</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>150018</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>337613</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Símbolo de &quot;Não Permitido&quot; 6">
+        <xdr:cNvPr id="12" name="Símbolo de &quot;Não Permitido&quot; 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{697F3794-D170-488C-9FA3-DF7D85C76F9F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D31F5258-D757-4BB9-B8B6-920EBBBD6A4C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5593,7 +5602,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9372444" y="997743"/>
+          <a:off x="3852338" y="809625"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5636,23 +5645,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>285594</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>45243</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>230050</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>390369</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>150018</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>334825</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="Símbolo de &quot;Não Permitido&quot; 7">
+        <xdr:cNvPr id="26" name="Símbolo de &quot;Não Permitido&quot; 25">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3B6F1BA-086A-408D-9091-583B7A5D7F21}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37A4F6F4-6DC0-424E-8762-26345C9CE02A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5660,7 +5669,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9381969" y="2140743"/>
+          <a:off x="3849550" y="1190625"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5703,23 +5712,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>276069</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>45243</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>247652</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>41413</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>380844</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>150018</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352427</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>146188</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="Símbolo de &quot;Não Permitido&quot; 8">
+        <xdr:cNvPr id="30" name="Símbolo de &quot;Não Permitido&quot; 29">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{042DDD9C-5EB5-4A26-A901-C54C9C5DF81A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1CE9C15D-5454-402E-83A9-27BA2F65C791}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5727,7 +5736,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9372444" y="1378743"/>
+          <a:off x="3867152" y="1755913"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5770,23 +5779,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>270116</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>51197</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>242889</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>50938</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>374891</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>155972</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>347664</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>155713</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="Símbolo de &quot;Não Permitido&quot; 9">
+        <xdr:cNvPr id="31" name="Símbolo de &quot;Não Permitido&quot; 30">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C12EDB1F-DE81-42F4-86F0-8E2A2F6E2231}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C76CD9F-0C8D-4A19-AAB6-101283051A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5794,7 +5803,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9366491" y="622697"/>
+          <a:off x="3862389" y="1574938"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5837,23 +5846,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>279641</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>51197</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>259948</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>384416</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>155972</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>364723</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Símbolo de &quot;Não Permitido&quot; 10">
+        <xdr:cNvPr id="32" name="Símbolo de &quot;Não Permitido&quot; 31">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F4A2CD1-AC5E-4A03-A73C-0837820A0A37}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5AD8321D-C6AB-47E4-949C-05976005D425}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5861,7 +5870,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9376016" y="1956197"/>
+          <a:off x="8121736" y="2133600"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5904,23 +5913,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>257685</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>240898</xdr:colOff>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>362460</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>345673</xdr:colOff>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="Símbolo de &quot;Não Permitido&quot; 11">
+        <xdr:cNvPr id="33" name="Símbolo de &quot;Não Permitido&quot; 32">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D31F5258-D757-4BB9-B8B6-920EBBBD6A4C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F73683A-5632-4538-A385-51A456178C1F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5928,7 +5937,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5086860" y="809625"/>
+          <a:off x="8102686" y="1381125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5971,23 +5980,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>274694</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>46159</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>245660</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>379469</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>150934</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>350435</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="Símbolo de &quot;Não Permitido&quot; 12">
+        <xdr:cNvPr id="34" name="Símbolo de &quot;Não Permitido&quot; 33">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30E782BB-A40A-4FC1-9BE9-732A014707E5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93813D1F-087D-41E3-857E-E47ECD0310D5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5995,7 +6004,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9371069" y="808159"/>
+          <a:off x="8107448" y="619125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6038,23 +6047,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>275811</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>61291</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>255185</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>380586</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>166066</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>359960</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="Símbolo de &quot;Não Permitido&quot; 13">
+        <xdr:cNvPr id="35" name="Símbolo de &quot;Não Permitido&quot; 34">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60376657-4A43-43D5-BEB0-BA3F2C81CA7C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A586073-1B38-4FF2-9FC8-0A0773A1CE36}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6062,7 +6071,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13639386" y="2156791"/>
+          <a:off x="8116973" y="1952625"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6105,23 +6114,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>256761</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>70816</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>245660</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>361536</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>175591</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>350435</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="Símbolo de &quot;Não Permitido&quot; 14">
+        <xdr:cNvPr id="36" name="Símbolo de &quot;Não Permitido&quot; 35">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6EED0F30-4718-402E-9831-D05D667B4EA5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05756E94-8483-443D-8644-5B0E9595CBB3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6129,7 +6138,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13620336" y="1404316"/>
+          <a:off x="8107448" y="1000125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6172,23 +6181,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>261523</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>70816</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>240165</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>366298</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>175591</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>344940</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="Símbolo de &quot;Não Permitido&quot; 15">
+        <xdr:cNvPr id="37" name="Símbolo de &quot;Não Permitido&quot; 36">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{53E18134-0F1B-4E6C-B228-B4DA01F5CCCB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F7B3695-CF9F-4AF2-8A18-5625270D1948}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6196,7 +6205,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13625098" y="642316"/>
+          <a:off x="8101953" y="809625"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6239,23 +6248,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>271048</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>70816</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>237377</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>375823</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>175591</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>342152</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="Símbolo de &quot;Não Permitido&quot; 16">
+        <xdr:cNvPr id="38" name="Símbolo de &quot;Não Permitido&quot; 37">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBE98AFE-8ED7-4AEA-9C3F-FAE47FFCAF91}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE4DC70A-5DAD-4AAD-A4E7-B407CC36B5B7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6263,7 +6272,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13634623" y="1975816"/>
+          <a:off x="8099165" y="1190625"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6306,23 +6315,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>261523</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>70816</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>254979</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>41413</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>366298</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>175591</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>359754</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>146188</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="Símbolo de &quot;Não Permitido&quot; 17">
+        <xdr:cNvPr id="39" name="Símbolo de &quot;Não Permitido&quot; 38">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58FE3CFE-9F69-4F6A-B901-3A428278A34D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44E7461E-D49C-4373-AFBE-BDF06B551B00}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6330,7 +6339,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13625098" y="1023316"/>
+          <a:off x="8116767" y="1755913"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6373,23 +6382,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>256028</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>70816</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>250216</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>50938</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>360803</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>175591</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>354991</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>155713</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="19" name="Símbolo de &quot;Não Permitido&quot; 18">
+        <xdr:cNvPr id="40" name="Símbolo de &quot;Não Permitido&quot; 39">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A2C3063-D2F6-415C-B36A-0D537EB4AABA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{335945EC-6C21-48E0-9716-244290DEEBAC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6397,7 +6406,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13619603" y="832816"/>
+          <a:off x="8112004" y="1574938"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6440,23 +6449,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>303973</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>273136</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>48039</xdr:rowOff>
+      <xdr:rowOff>43961</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>408748</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>377911</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>152814</xdr:rowOff>
+      <xdr:rowOff>148736</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="20" name="Símbolo de &quot;Não Permitido&quot; 19">
+        <xdr:cNvPr id="41" name="Símbolo de &quot;Não Permitido&quot; 40">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF856C43-FDCB-451D-8B8D-DD79F0988083}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61B7E8D9-D880-43E3-B441-59065E9460BD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6464,7 +6473,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17934748" y="2143539"/>
+          <a:off x="12391867" y="2139461"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6507,23 +6516,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>284923</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>254086</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>57564</xdr:rowOff>
+      <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>389698</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>358861</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>162339</xdr:rowOff>
+      <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="Símbolo de &quot;Não Permitido&quot; 20">
+        <xdr:cNvPr id="42" name="Símbolo de &quot;Não Permitido&quot; 41">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{933FA514-839A-497A-AF7C-96FD9F783A29}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90AFAF4D-7CBB-4DE9-82FB-DC3E81A1A892}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6531,7 +6540,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17915698" y="1391064"/>
+          <a:off x="12372817" y="1386986"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6574,23 +6583,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>289685</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>258848</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>57564</xdr:rowOff>
+      <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>394460</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>363623</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>162339</xdr:rowOff>
+      <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="Símbolo de &quot;Não Permitido&quot; 21">
+        <xdr:cNvPr id="43" name="Símbolo de &quot;Não Permitido&quot; 42">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CF93C78-BABA-4E57-810A-C090AB2871CD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDA51E2E-C6A2-4549-A46E-0E5E59645B8F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6598,7 +6607,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17920460" y="629064"/>
+          <a:off x="12377579" y="624986"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6641,23 +6650,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>299210</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>268373</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>57564</xdr:rowOff>
+      <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>403985</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>373148</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>162339</xdr:rowOff>
+      <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="Símbolo de &quot;Não Permitido&quot; 22">
+        <xdr:cNvPr id="44" name="Símbolo de &quot;Não Permitido&quot; 43">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4380C4F6-AD10-4A14-8F21-989FC1B7D363}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A80B2AD2-6F5E-4AC5-B4B7-F98C7765AC82}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6665,7 +6674,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17929985" y="1962564"/>
+          <a:off x="12387104" y="1958486"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6708,23 +6717,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>289685</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>258848</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>57564</xdr:rowOff>
+      <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>394460</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>363623</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>162339</xdr:rowOff>
+      <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="Símbolo de &quot;Não Permitido&quot; 23">
+        <xdr:cNvPr id="45" name="Símbolo de &quot;Não Permitido&quot; 44">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFA6B7CB-6C94-4117-A552-83D2018E738A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DBDB679-27EB-4E48-A937-3DAA9D1368D6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6732,7 +6741,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17920460" y="1010064"/>
+          <a:off x="12377579" y="1005986"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6775,23 +6784,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>284190</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>253353</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>57564</xdr:rowOff>
+      <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>388965</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>358128</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>162339</xdr:rowOff>
+      <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="Símbolo de &quot;Não Permitido&quot; 24">
+        <xdr:cNvPr id="46" name="Símbolo de &quot;Não Permitido&quot; 45">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27DD8CD5-DB8D-47EB-8EBF-FCBD5AEAED2F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A193B186-603F-4FB5-B303-222457EED99E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6799,7 +6808,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="17914965" y="819564"/>
+          <a:off x="12372084" y="815486"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6842,23 +6851,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>254897</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>250565</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>359672</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>355340</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="Símbolo de &quot;Não Permitido&quot; 25">
+        <xdr:cNvPr id="47" name="Símbolo de &quot;Não Permitido&quot; 46">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37A4F6F4-6DC0-424E-8762-26345C9CE02A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB622CA5-ED9C-4DA1-9AFA-53C533AF7C4B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6866,7 +6875,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5084072" y="1190625"/>
+          <a:off x="12369296" y="1196486"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6909,23 +6918,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>266493</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>42656</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>268167</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>47274</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>371268</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>147431</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>372942</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>152049</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="Símbolo de &quot;Não Permitido&quot; 26">
+        <xdr:cNvPr id="48" name="Símbolo de &quot;Não Permitido&quot; 47">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11609110-43B1-4A51-9932-8CBF37AD6A8E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E12E6F4B-1B58-4296-9C49-AE0AC40CBE30}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6933,7 +6942,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9362868" y="1185656"/>
+          <a:off x="12386898" y="1761774"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6976,23 +6985,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>269806</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>45969</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>263404</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>56799</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>374581</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>150744</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>368179</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>161574</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="Símbolo de &quot;Não Permitido&quot; 27">
+        <xdr:cNvPr id="49" name="Símbolo de &quot;Não Permitido&quot; 48">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11839849-9983-4F57-B67E-E5088CBAFB96}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82A7787B-D6D5-4D82-80A0-FF505FBEB437}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7000,7 +7009,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13633381" y="1188969"/>
+          <a:off x="12382135" y="1580799"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -7043,23 +7052,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>256761</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>62533</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>257018</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>49823</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>361536</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>167308</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>361793</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>154598</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="Símbolo de &quot;Não Permitido&quot; 28">
+        <xdr:cNvPr id="50" name="Símbolo de &quot;Não Permitido&quot; 49">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDA9C6B7-CD65-4DC5-986F-9553C21D9FFD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5ACE145-5B20-4D33-B7D4-75D298F98632}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7067,7 +7076,543 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13620336" y="1586533"/>
+          <a:off x="16632691" y="2145323"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>237968</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>59348</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>342743</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>164123</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="51" name="Símbolo de &quot;Não Permitido&quot; 50">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A42EFB1D-D430-4B59-8412-C091DF0FBA93}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16613641" y="1392848"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>242730</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>59348</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>347505</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>164123</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="52" name="Símbolo de &quot;Não Permitido&quot; 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25002C19-F5C9-4FDA-A571-7581DC00C285}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16618403" y="630848"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>252255</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>59348</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>357030</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>164123</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="Símbolo de &quot;Não Permitido&quot; 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E08C98E7-8F45-47B8-8EBD-C099EC3508E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16627928" y="1964348"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>242730</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>59348</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>347505</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>164123</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="54" name="Símbolo de &quot;Não Permitido&quot; 53">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CCDCF4B7-440F-4F55-B7E2-1457A1790821}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16618403" y="1011848"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>237235</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>59348</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>342010</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>164123</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="55" name="Símbolo de &quot;Não Permitido&quot; 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25844D48-AE20-42B0-AEB6-B39797162158}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16612908" y="821348"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>234447</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>59348</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>339222</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>164123</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="56" name="Símbolo de &quot;Não Permitido&quot; 55">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1E11017-880E-4384-8E9A-DB6C6F5BB75F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16610120" y="1202348"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>252049</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>53136</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>356824</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>157911</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="Símbolo de &quot;Não Permitido&quot; 56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{053B77BD-4750-42CC-95BA-5720144C0B64}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16627722" y="1767636"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>247286</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>62661</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>352061</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>167436</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="58" name="Símbolo de &quot;Não Permitido&quot; 57">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49A075DE-2A6D-4A19-8BA2-F0EF72ECB970}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16622959" y="1586661"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -9953,887 +10498,446 @@
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" s="109"/>
       <c r="B3" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="H3" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="I3" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="J3" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="K3" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="L3" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="M3" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="N3" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="50" t="s">
+      <c r="O3" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="50" t="s">
+      <c r="P3" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="50" t="s">
+      <c r="Q3" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="M3" s="50" t="s">
+      <c r="R3" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="N3" s="50" t="s">
+      <c r="S3" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="50" t="s">
+      <c r="T3" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="50" t="s">
+      <c r="U3" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="50" t="s">
+      <c r="V3" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="50" t="s">
+      <c r="W3" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="50" t="s">
+      <c r="X3" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="T3" s="50" t="s">
+      <c r="Y3" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="U3" s="50" t="s">
+      <c r="Z3" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="V3" s="50" t="s">
+      <c r="AA3" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="50" t="s">
+      <c r="AB3" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="X3" s="50" t="s">
+      <c r="AC3" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="Y3" s="50" t="s">
+      <c r="AD3" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="Z3" s="50" t="s">
+      <c r="AE3" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="AA3" s="50" t="s">
+      <c r="AF3" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="AB3" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC3" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="AD3" s="50" t="s">
-        <v>18</v>
-      </c>
-      <c r="AE3" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="AF3" s="50"/>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="36">
-        <v>7400</v>
-      </c>
-      <c r="C4" s="36">
-        <v>2290</v>
-      </c>
-      <c r="D4" s="36">
-        <v>27210</v>
-      </c>
-      <c r="E4" s="36">
-        <v>4390</v>
-      </c>
-      <c r="F4" s="36">
-        <v>1240</v>
-      </c>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
       <c r="G4" s="36"/>
-      <c r="H4" s="74" t="s">
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="36">
-        <v>4820</v>
-      </c>
-      <c r="J4" s="36">
-        <v>15570</v>
-      </c>
-      <c r="K4" s="36">
-        <v>1660</v>
-      </c>
-      <c r="L4" s="46">
-        <v>16310</v>
-      </c>
-      <c r="M4" s="1"/>
       <c r="N4" s="1"/>
-      <c r="O4" s="8">
-        <v>4230</v>
-      </c>
-      <c r="P4" s="8">
-        <v>10240</v>
-      </c>
-      <c r="Q4" s="8">
-        <v>2880</v>
-      </c>
-      <c r="R4" s="46">
-        <v>7900</v>
-      </c>
-      <c r="S4" s="46">
-        <v>4420</v>
-      </c>
-      <c r="T4" s="46">
-        <v>13220</v>
-      </c>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="46"/>
+      <c r="S4" s="46"/>
+      <c r="T4" s="46"/>
       <c r="U4" s="36"/>
-      <c r="V4" s="46">
-        <v>11440</v>
-      </c>
-      <c r="W4" s="46">
-        <v>2770</v>
-      </c>
-      <c r="X4" s="8">
-        <v>11640</v>
-      </c>
-      <c r="Y4" s="36">
-        <v>3260</v>
-      </c>
-      <c r="Z4" s="36">
-        <v>23410</v>
-      </c>
-      <c r="AA4" s="36">
-        <v>1470</v>
-      </c>
+      <c r="V4" s="46"/>
+      <c r="W4" s="46"/>
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="36"/>
       <c r="AB4" s="36"/>
-      <c r="AC4" s="36">
-        <v>4740</v>
-      </c>
-      <c r="AD4" s="36">
-        <v>11450</v>
-      </c>
-      <c r="AE4" s="8">
-        <v>4950</v>
-      </c>
-      <c r="AF4" s="49"/>
+      <c r="AC4" s="36"/>
+      <c r="AD4" s="36"/>
+      <c r="AE4" s="36"/>
+      <c r="AF4" s="36"/>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="36">
-        <v>203220</v>
-      </c>
-      <c r="C5" s="8">
-        <v>160240</v>
-      </c>
-      <c r="D5" s="36">
-        <v>155770</v>
-      </c>
-      <c r="E5" s="36">
-        <v>147150</v>
-      </c>
-      <c r="F5" s="36">
-        <v>98380</v>
-      </c>
+      <c r="B5" s="36"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
       <c r="G5" s="36"/>
-      <c r="H5" s="74" t="s">
+      <c r="H5" s="36"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="36">
-        <v>224420</v>
-      </c>
-      <c r="J5" s="8">
-        <v>154910</v>
-      </c>
-      <c r="K5" s="8">
-        <v>163080</v>
-      </c>
-      <c r="L5" s="36">
-        <v>148320</v>
-      </c>
-      <c r="M5" s="8"/>
       <c r="N5" s="8"/>
-      <c r="O5" s="8">
-        <v>181980</v>
-      </c>
-      <c r="P5" s="8">
-        <v>172160</v>
-      </c>
-      <c r="Q5" s="8">
-        <v>118500</v>
-      </c>
-      <c r="R5" s="40">
-        <v>179190</v>
-      </c>
-      <c r="S5" s="36">
-        <v>125350</v>
-      </c>
-      <c r="T5" s="36">
-        <v>54020</v>
-      </c>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="36"/>
+      <c r="R5" s="40"/>
+      <c r="S5" s="36"/>
+      <c r="T5" s="36"/>
       <c r="U5" s="36"/>
-      <c r="V5" s="36">
-        <v>290700</v>
-      </c>
-      <c r="W5" s="36">
-        <v>241680</v>
-      </c>
-      <c r="X5" s="8">
-        <v>228200</v>
-      </c>
-      <c r="Y5" s="36">
-        <v>235220</v>
-      </c>
-      <c r="Z5" s="36">
-        <v>326450</v>
-      </c>
-      <c r="AA5" s="36">
-        <v>80060</v>
-      </c>
+      <c r="V5" s="36"/>
+      <c r="W5" s="36"/>
+      <c r="X5" s="36"/>
+      <c r="Y5" s="36"/>
+      <c r="Z5" s="36"/>
+      <c r="AA5" s="36"/>
       <c r="AB5" s="40"/>
-      <c r="AC5" s="36">
-        <v>203590</v>
-      </c>
-      <c r="AD5" s="36">
-        <v>206570</v>
-      </c>
-      <c r="AE5" s="8">
-        <v>171260</v>
-      </c>
-      <c r="AF5" s="49"/>
+      <c r="AC5" s="36"/>
+      <c r="AD5" s="36"/>
+      <c r="AE5" s="36"/>
+      <c r="AF5" s="36"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="36">
-        <v>170020</v>
-      </c>
-      <c r="C6" s="8">
-        <v>96730</v>
-      </c>
-      <c r="D6" s="36">
-        <v>98520</v>
-      </c>
-      <c r="E6" s="36">
-        <v>96940</v>
-      </c>
-      <c r="F6" s="36">
-        <v>105120</v>
-      </c>
+      <c r="B6" s="36"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
       <c r="G6" s="36"/>
-      <c r="H6" s="74">
-        <v>94920</v>
-      </c>
-      <c r="I6" s="36">
-        <v>119340</v>
-      </c>
-      <c r="J6" s="8">
-        <v>115580</v>
-      </c>
-      <c r="K6" s="8">
-        <v>87050</v>
-      </c>
-      <c r="L6" s="36">
-        <v>101530</v>
-      </c>
-      <c r="M6" s="8"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="121" t="s">
+        <v>23</v>
+      </c>
       <c r="N6" s="8"/>
-      <c r="O6" s="8">
-        <v>95630</v>
-      </c>
-      <c r="P6" s="9">
-        <v>153720</v>
-      </c>
-      <c r="Q6" s="8">
-        <v>80250</v>
-      </c>
-      <c r="R6" s="36">
-        <v>103290</v>
-      </c>
-      <c r="S6" s="36">
-        <v>67600</v>
-      </c>
-      <c r="T6" s="36">
-        <v>113370</v>
-      </c>
+      <c r="O6" s="36"/>
+      <c r="P6" s="119"/>
+      <c r="Q6" s="36"/>
+      <c r="R6" s="36"/>
+      <c r="S6" s="36"/>
+      <c r="T6" s="36"/>
       <c r="U6" s="36"/>
-      <c r="V6" s="36">
-        <v>90830</v>
-      </c>
-      <c r="W6" s="36">
-        <v>142100</v>
-      </c>
-      <c r="X6" s="8">
-        <v>67060</v>
-      </c>
-      <c r="Y6" s="36">
-        <v>85360</v>
-      </c>
-      <c r="Z6" s="36">
-        <v>98480</v>
-      </c>
-      <c r="AA6" s="36">
-        <v>78770</v>
-      </c>
+      <c r="V6" s="36"/>
+      <c r="W6" s="36"/>
+      <c r="X6" s="36"/>
+      <c r="Y6" s="36"/>
+      <c r="Z6" s="36"/>
+      <c r="AA6" s="36"/>
       <c r="AB6" s="36"/>
-      <c r="AC6" s="36">
-        <v>89170</v>
-      </c>
-      <c r="AD6" s="36">
-        <v>142000</v>
-      </c>
-      <c r="AE6" s="8">
-        <v>75050</v>
-      </c>
-      <c r="AF6" s="49"/>
+      <c r="AC6" s="36"/>
+      <c r="AD6" s="36"/>
+      <c r="AE6" s="36"/>
+      <c r="AF6" s="36"/>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="36">
-        <f>(B6*(1-($B$46)))</f>
-        <v>151317.79999999999</v>
-      </c>
-      <c r="C7" s="36">
-        <f>(C6*(1-($B$46)))</f>
-        <v>86089.7</v>
-      </c>
-      <c r="D7" s="36">
-        <f>(D6*(1-($B$46)))</f>
-        <v>87682.8</v>
-      </c>
-      <c r="E7" s="36">
-        <f>(E6*(1-($B$46)))</f>
-        <v>86276.6</v>
-      </c>
-      <c r="F7" s="36">
-        <f>(F6*(1-($B$46)))</f>
-        <v>93556.800000000003</v>
-      </c>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
       <c r="G7" s="36"/>
-      <c r="H7" s="74">
-        <f t="shared" ref="H7:L7" si="0">(H6*(1-($B$46)))</f>
-        <v>84478.8</v>
-      </c>
-      <c r="I7" s="36">
-        <f t="shared" si="0"/>
-        <v>106212.6</v>
-      </c>
-      <c r="J7" s="36">
-        <f t="shared" si="0"/>
-        <v>102866.2</v>
-      </c>
-      <c r="K7" s="36">
-        <f t="shared" si="0"/>
-        <v>77474.5</v>
-      </c>
-      <c r="L7" s="36">
-        <f t="shared" si="0"/>
-        <v>90361.7</v>
-      </c>
-      <c r="M7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="36"/>
+      <c r="L7" s="36"/>
+      <c r="M7" s="121" t="s">
+        <v>23</v>
+      </c>
       <c r="N7" s="36"/>
-      <c r="O7" s="82">
-        <v>95630</v>
-      </c>
-      <c r="P7" s="83">
-        <v>153720</v>
-      </c>
-      <c r="Q7" s="82">
-        <f t="shared" ref="Q7:R7" si="1">(Q6-(Q9-Q10))</f>
-        <v>80161.403999999995</v>
-      </c>
-      <c r="R7" s="82">
-        <f t="shared" si="1"/>
-        <v>103199.15</v>
-      </c>
-      <c r="S7" s="82">
-        <f>(S6-(S9-S10))</f>
-        <v>67511.127999999997</v>
-      </c>
-      <c r="T7" s="36">
-        <v>113370</v>
-      </c>
+      <c r="O7" s="36"/>
+      <c r="P7" s="119"/>
+      <c r="Q7" s="36"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="36"/>
+      <c r="T7" s="36"/>
       <c r="U7" s="36"/>
-      <c r="V7" s="36">
-        <f>(V6-(V9-V10))</f>
-        <v>88599.2</v>
-      </c>
-      <c r="W7" s="36">
-        <f t="shared" ref="W7:Y7" si="2">(W6-(W9-W10))</f>
-        <v>139964.9</v>
-      </c>
-      <c r="X7" s="36">
-        <f t="shared" si="2"/>
-        <v>65192.2</v>
-      </c>
-      <c r="Y7" s="36">
-        <f t="shared" si="2"/>
-        <v>82919.100000000006</v>
-      </c>
-      <c r="Z7" s="36">
-        <f>(Z6-(Z9-Z10))</f>
-        <v>96597.9</v>
-      </c>
+      <c r="V7" s="36"/>
+      <c r="W7" s="36"/>
+      <c r="X7" s="36"/>
+      <c r="Y7" s="36"/>
+      <c r="Z7" s="36"/>
       <c r="AA7" s="36"/>
       <c r="AB7" s="36"/>
-      <c r="AC7" s="36">
-        <f t="shared" ref="AC7:AE7" si="3">(AC6-(AC9-AC10))</f>
-        <v>86962.3</v>
-      </c>
-      <c r="AD7" s="36">
-        <f t="shared" si="3"/>
-        <v>139952.9</v>
-      </c>
-      <c r="AE7" s="36">
-        <f t="shared" si="3"/>
-        <v>72743.3</v>
-      </c>
-      <c r="AF7" s="49"/>
+      <c r="AC7" s="36"/>
+      <c r="AD7" s="36"/>
+      <c r="AE7" s="36"/>
+      <c r="AF7" s="36"/>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="47">
-        <v>450</v>
-      </c>
-      <c r="C8" s="8">
-        <v>560</v>
-      </c>
-      <c r="D8" s="47">
-        <v>510</v>
-      </c>
-      <c r="E8" s="47">
-        <v>590</v>
-      </c>
-      <c r="F8" s="47">
-        <v>380</v>
-      </c>
+      <c r="B8" s="47"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="47"/>
       <c r="G8" s="47"/>
-      <c r="H8" s="75">
-        <v>2810</v>
-      </c>
-      <c r="I8" s="47">
-        <v>340</v>
-      </c>
-      <c r="J8" s="8">
-        <v>420</v>
-      </c>
-      <c r="K8" s="10">
-        <v>690</v>
-      </c>
-      <c r="L8" s="47">
-        <v>670</v>
-      </c>
-      <c r="M8" s="10"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="47"/>
+      <c r="J8" s="36"/>
+      <c r="K8" s="47"/>
+      <c r="L8" s="47"/>
+      <c r="M8" s="121" t="s">
+        <v>23</v>
+      </c>
       <c r="N8" s="8"/>
-      <c r="O8" s="8">
-        <v>890</v>
-      </c>
-      <c r="P8" s="9">
-        <v>560</v>
-      </c>
-      <c r="Q8" s="8">
-        <v>500</v>
-      </c>
-      <c r="R8" s="36">
-        <v>0</v>
-      </c>
-      <c r="S8" s="36">
-        <v>1680</v>
-      </c>
+      <c r="O8" s="36"/>
+      <c r="P8" s="119"/>
+      <c r="Q8" s="36"/>
+      <c r="R8" s="36"/>
+      <c r="S8" s="36"/>
       <c r="T8" s="36"/>
       <c r="U8" s="26"/>
-      <c r="V8" s="36">
-        <v>440</v>
-      </c>
-      <c r="W8" s="36">
-        <v>420</v>
-      </c>
-      <c r="X8" s="8">
-        <v>510</v>
-      </c>
-      <c r="Y8" s="36">
-        <v>370</v>
-      </c>
-      <c r="Z8" s="36">
-        <v>3020</v>
-      </c>
-      <c r="AA8" s="36">
-        <v>640</v>
-      </c>
+      <c r="V8" s="36"/>
+      <c r="W8" s="36"/>
+      <c r="X8" s="36"/>
+      <c r="Y8" s="36"/>
+      <c r="Z8" s="36"/>
+      <c r="AA8" s="36"/>
       <c r="AB8" s="36"/>
-      <c r="AC8" s="36">
-        <v>400</v>
-      </c>
-      <c r="AD8" s="36">
-        <v>920</v>
-      </c>
-      <c r="AE8" s="8">
-        <v>230</v>
-      </c>
-      <c r="AF8" s="49"/>
+      <c r="AC8" s="36"/>
+      <c r="AD8" s="36"/>
+      <c r="AE8" s="36"/>
+      <c r="AF8" s="36"/>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" s="84" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="47">
-        <v>21490</v>
-      </c>
-      <c r="C9" s="8">
-        <v>19540</v>
-      </c>
-      <c r="D9" s="47">
-        <v>23760</v>
-      </c>
-      <c r="E9" s="47">
-        <v>21110</v>
-      </c>
+      <c r="B9" s="47"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
       <c r="F9" s="47"/>
       <c r="G9" s="47"/>
-      <c r="H9" s="76" t="s">
+      <c r="H9" s="120"/>
+      <c r="I9" s="47"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="36"/>
+      <c r="L9" s="47"/>
+      <c r="M9" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="47">
-        <v>19080</v>
-      </c>
-      <c r="J9" s="47">
-        <v>22440</v>
-      </c>
-      <c r="K9" s="8">
-        <v>19090</v>
-      </c>
-      <c r="L9" s="47">
-        <v>21720</v>
-      </c>
-      <c r="M9" s="10"/>
       <c r="N9" s="8"/>
-      <c r="O9" s="8">
-        <v>26570</v>
-      </c>
-      <c r="P9" s="8">
-        <v>21070</v>
-      </c>
-      <c r="Q9" s="8">
-        <v>19260</v>
-      </c>
-      <c r="R9" s="36">
-        <v>19750</v>
-      </c>
-      <c r="S9" s="36">
-        <v>19320</v>
-      </c>
+      <c r="O9" s="36"/>
+      <c r="P9" s="36"/>
+      <c r="Q9" s="36"/>
+      <c r="R9" s="36"/>
+      <c r="S9" s="36"/>
       <c r="T9" s="36"/>
       <c r="U9" s="26"/>
-      <c r="V9" s="36">
-        <v>20280</v>
-      </c>
-      <c r="W9" s="36">
-        <v>19410</v>
-      </c>
-      <c r="X9" s="8">
-        <v>16980</v>
-      </c>
-      <c r="Y9" s="36">
-        <v>22190</v>
-      </c>
-      <c r="Z9" s="36">
-        <v>17110</v>
-      </c>
+      <c r="V9" s="36"/>
+      <c r="W9" s="36"/>
+      <c r="X9" s="36"/>
+      <c r="Y9" s="36"/>
+      <c r="Z9" s="36"/>
       <c r="AA9" s="36"/>
       <c r="AB9" s="36"/>
-      <c r="AC9" s="36">
-        <v>20070</v>
-      </c>
-      <c r="AD9" s="36">
-        <v>18610</v>
-      </c>
-      <c r="AE9" s="8">
-        <v>20970</v>
-      </c>
-      <c r="AF9" s="49"/>
+      <c r="AC9" s="36"/>
+      <c r="AD9" s="36"/>
+      <c r="AE9" s="36"/>
+      <c r="AF9" s="36"/>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="47">
-        <f>(B9*(1-($B$46)))</f>
-        <v>19126.099999999999</v>
-      </c>
-      <c r="C10" s="47">
-        <f t="shared" ref="C10:L10" si="4">(C9*(1-($B$46)))</f>
-        <v>17390.599999999999</v>
-      </c>
-      <c r="D10" s="47">
-        <f t="shared" si="4"/>
-        <v>21146.400000000001</v>
-      </c>
-      <c r="E10" s="47">
-        <f t="shared" si="4"/>
-        <v>18787.900000000001</v>
-      </c>
-      <c r="F10" s="47">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
       <c r="G10" s="47"/>
-      <c r="H10" s="77" t="s">
+      <c r="H10" s="46"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
+      <c r="K10" s="47"/>
+      <c r="L10" s="47"/>
+      <c r="M10" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="47">
-        <f t="shared" si="4"/>
-        <v>16981.2</v>
-      </c>
-      <c r="J10" s="47">
-        <f t="shared" si="4"/>
-        <v>19971.599999999999</v>
-      </c>
-      <c r="K10" s="47">
-        <f t="shared" si="4"/>
-        <v>16990.099999999999</v>
-      </c>
-      <c r="L10" s="47">
-        <f t="shared" si="4"/>
-        <v>19330.8</v>
-      </c>
-      <c r="M10" s="10"/>
       <c r="N10" s="8"/>
-      <c r="O10" s="69" t="s">
-        <v>52</v>
-      </c>
-      <c r="P10" s="69" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q10" s="47">
-        <f>(Q9*(1-($E$46)))</f>
-        <v>19171.403999999999</v>
-      </c>
-      <c r="R10" s="47">
-        <f t="shared" ref="R10:T10" si="5">(R9*(1-($E$46)))</f>
-        <v>19659.149999999998</v>
-      </c>
-      <c r="S10" s="47">
-        <f t="shared" si="5"/>
-        <v>19231.128000000001</v>
-      </c>
-      <c r="T10" s="47">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
+      <c r="O10" s="47"/>
+      <c r="P10" s="47"/>
+      <c r="Q10" s="47"/>
+      <c r="R10" s="47"/>
+      <c r="S10" s="47"/>
+      <c r="T10" s="47"/>
       <c r="U10" s="47"/>
-      <c r="V10" s="47">
-        <f>(V9*(1-($C$46)))</f>
-        <v>18049.2</v>
-      </c>
-      <c r="W10" s="47">
-        <f t="shared" ref="W10:AE10" si="6">(W9*(1-($C$46)))</f>
-        <v>17274.900000000001</v>
-      </c>
-      <c r="X10" s="47">
-        <f t="shared" si="6"/>
-        <v>15112.2</v>
-      </c>
-      <c r="Y10" s="47">
-        <f t="shared" si="6"/>
-        <v>19749.099999999999</v>
-      </c>
-      <c r="Z10" s="47">
-        <f t="shared" si="6"/>
-        <v>15227.9</v>
-      </c>
+      <c r="V10" s="47"/>
+      <c r="W10" s="47"/>
+      <c r="X10" s="47"/>
+      <c r="Y10" s="47"/>
+      <c r="Z10" s="47"/>
       <c r="AA10" s="47"/>
       <c r="AB10" s="47"/>
-      <c r="AC10" s="47">
-        <f t="shared" si="6"/>
-        <v>17862.3</v>
-      </c>
-      <c r="AD10" s="47">
-        <f t="shared" si="6"/>
-        <v>16562.900000000001</v>
-      </c>
-      <c r="AE10" s="47">
-        <f t="shared" si="6"/>
-        <v>18663.3</v>
-      </c>
-      <c r="AF10" s="49"/>
+      <c r="AC10" s="47"/>
+      <c r="AD10" s="47"/>
+      <c r="AE10" s="47"/>
+      <c r="AF10" s="36"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="36">
-        <v>604800</v>
-      </c>
-      <c r="C11" s="8">
-        <v>126000</v>
-      </c>
-      <c r="D11" s="36">
-        <v>403200</v>
-      </c>
-      <c r="E11" s="36">
-        <v>201600</v>
-      </c>
+      <c r="B11" s="36"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
       <c r="F11" s="36"/>
       <c r="G11" s="36"/>
-      <c r="H11" s="74" t="s">
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="36"/>
+      <c r="L11" s="36"/>
+      <c r="M11" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="I11" s="36">
-        <v>403200</v>
-      </c>
-      <c r="J11" s="36">
-        <v>403200</v>
-      </c>
-      <c r="K11" s="8">
-        <v>181440</v>
-      </c>
-      <c r="L11" s="36">
-        <v>352800</v>
-      </c>
-      <c r="M11" s="8"/>
       <c r="N11" s="8"/>
-      <c r="O11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="P11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="R11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="S11" s="33" t="s">
-        <v>53</v>
-      </c>
+      <c r="O11" s="36"/>
+      <c r="P11" s="36"/>
+      <c r="Q11" s="36"/>
+      <c r="R11" s="36"/>
+      <c r="S11" s="36"/>
       <c r="T11" s="36"/>
       <c r="U11" s="36"/>
-      <c r="V11" s="36">
-        <v>201600</v>
-      </c>
-      <c r="W11" s="36">
-        <v>302400</v>
-      </c>
-      <c r="X11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z11" s="33" t="s">
-        <v>53</v>
-      </c>
+      <c r="V11" s="36"/>
+      <c r="W11" s="36"/>
+      <c r="X11" s="36"/>
+      <c r="Y11" s="36"/>
+      <c r="Z11" s="36"/>
       <c r="AA11" s="36"/>
       <c r="AB11" s="36"/>
-      <c r="AC11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="AF11" s="49"/>
+      <c r="AC11" s="36"/>
+      <c r="AD11" s="36"/>
+      <c r="AE11" s="36"/>
+      <c r="AF11" s="36"/>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" s="73" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="36"/>
-      <c r="C12" s="8">
-        <v>30000</v>
-      </c>
+      <c r="C12" s="8"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="36">
-        <v>30000</v>
-      </c>
+      <c r="E12" s="36"/>
       <c r="F12" s="36"/>
       <c r="G12" s="36"/>
-      <c r="H12" s="74" t="s">
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="36"/>
+      <c r="M12" s="121" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="J12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="K12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="L12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="M12" s="36"/>
       <c r="N12" s="8"/>
-      <c r="O12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="P12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="R12" s="36" t="s">
-        <v>51</v>
-      </c>
-      <c r="S12" s="30">
-        <v>20000</v>
-      </c>
+      <c r="O12" s="36"/>
+      <c r="P12" s="36"/>
+      <c r="Q12" s="36"/>
+      <c r="R12" s="36"/>
+      <c r="S12" s="36"/>
       <c r="T12" s="36"/>
       <c r="U12" s="36"/>
       <c r="V12" s="36"/>
-      <c r="W12" s="36">
-        <v>20000</v>
-      </c>
-      <c r="X12" s="8"/>
+      <c r="W12" s="36"/>
+      <c r="X12" s="36"/>
       <c r="Y12" s="36"/>
-      <c r="Z12" s="33" t="s">
-        <v>61</v>
-      </c>
+      <c r="Z12" s="36"/>
       <c r="AA12" s="36"/>
       <c r="AB12" s="36"/>
-      <c r="AC12" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="AD12" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="AE12" s="33" t="s">
-        <v>61</v>
-      </c>
-      <c r="AF12" s="49"/>
+      <c r="AC12" s="36"/>
+      <c r="AD12" s="36"/>
+      <c r="AE12" s="36"/>
+      <c r="AF12" s="36"/>
     </row>
     <row r="13" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="59"/>
       <c r="B13" s="60"/>
       <c r="C13" s="61"/>
       <c r="D13" s="62"/>
-      <c r="E13" s="78">
-        <v>273353</v>
-      </c>
       <c r="F13" s="62"/>
       <c r="G13" s="62"/>
       <c r="H13" s="62"/>
@@ -10847,15 +10951,9 @@
       <c r="P13" s="72"/>
       <c r="Q13" s="72"/>
       <c r="R13" s="62"/>
-      <c r="S13" s="78">
-        <v>273434</v>
-      </c>
       <c r="T13" s="62"/>
       <c r="U13" s="62"/>
       <c r="V13" s="62"/>
-      <c r="W13" s="78">
-        <v>273455</v>
-      </c>
       <c r="X13" s="61"/>
       <c r="Y13" s="62"/>
       <c r="Z13" s="62"/>
@@ -10864,7 +10962,6 @@
       <c r="AC13" s="62"/>
       <c r="AD13" s="62"/>
       <c r="AE13" s="61"/>
-      <c r="AF13" s="63"/>
     </row>
     <row r="14" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17"/>
@@ -10883,7 +10980,7 @@
       </c>
       <c r="B15" s="12">
         <f>SUM(B4:AF4)</f>
-        <v>198910</v>
+        <v>0</v>
       </c>
       <c r="J15" s="110" t="s">
         <v>45</v>
@@ -10897,7 +10994,7 @@
       </c>
       <c r="B16" s="12">
         <f>SUM(B5:AF5)</f>
-        <v>4270420</v>
+        <v>0</v>
       </c>
       <c r="J16" s="101" t="s">
         <v>46</v>
@@ -10921,7 +11018,7 @@
       </c>
       <c r="B17" s="12">
         <f>SUM(B6:AF6)</f>
-        <v>2568430</v>
+        <v>0</v>
       </c>
       <c r="J17" s="102" t="s">
         <v>48</v>
@@ -10947,7 +11044,7 @@
       </c>
       <c r="B18" s="12">
         <f>SUM(B7:AF7)</f>
-        <v>2352840.9819999994</v>
+        <v>0</v>
       </c>
       <c r="J18" s="101" t="s">
         <v>47</v>
@@ -10971,7 +11068,7 @@
       </c>
       <c r="B19" s="12">
         <f>SUM(B8:AF8)</f>
-        <v>18000</v>
+        <v>0</v>
       </c>
       <c r="J19" s="111" t="s">
         <v>49</v>
@@ -10987,8 +11084,8 @@
         <v>3</v>
       </c>
       <c r="B20" s="12">
-        <f t="shared" ref="B20:B21" si="7">SUM(B11:AF11)</f>
-        <v>3180240</v>
+        <f t="shared" ref="B20:B21" si="0">SUM(B11:AF11)</f>
+        <v>0</v>
       </c>
       <c r="J20" s="101" t="s">
         <v>50</v>
@@ -11003,8 +11100,8 @@
         <v>4</v>
       </c>
       <c r="B21" s="16">
-        <f t="shared" si="7"/>
-        <v>100000</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="R21" s="112"/>
       <c r="S21" s="112"/>
@@ -11277,6 +11374,7 @@
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="A39:E39"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
Atualiza dados da planilha da balanca (ate dia 15 de Outubro)
</commit_message>
<xml_diff>
--- a/BALANÇA_ATERRO.xlsx
+++ b/BALANÇA_ATERRO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muril\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44FACFD-D991-4826-B4E5-5AC19106AD2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50C452A8-1ED8-40CC-B3CC-214C7073639A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{DDC835EE-E68E-4405-84CA-BBF9A30D9944}"/>
+    <workbookView xWindow="510" yWindow="3300" windowWidth="13125" windowHeight="9465" activeTab="2" xr2:uid="{DDC835EE-E68E-4405-84CA-BBF9A30D9944}"/>
   </bookViews>
   <sheets>
     <sheet name="AGOSTO" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="66">
   <si>
     <t>Entulho</t>
   </si>
@@ -226,12 +226,25 @@
   <si>
     <t>Pipa Mant.</t>
   </si>
+  <si>
+    <t>Lixo Domiciliar (Coleta)</t>
+  </si>
+  <si>
+    <t>OUTUBRO (PESO EM KG)</t>
+  </si>
+  <si>
+    <t>PREÇO DO COMBUSTIVEL (R$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apenas 6 caminhões por dia vão para o cootcrat, a porcentagem deve ser contabilizada pela diferença do n reciclado, </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
@@ -283,7 +296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -374,8 +387,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="41">
+  <borders count="45">
     <border>
       <left/>
       <right/>
@@ -887,12 +906,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1017,6 +1085,27 @@
     <xf numFmtId="3" fontId="0" fillId="14" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1060,6 +1149,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1107,24 +1205,76 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Moeda" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -5245,13 +5395,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>252621</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>357396</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5312,13 +5462,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>233571</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>338346</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5446,13 +5596,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>247858</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>352633</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5514,13 +5664,13 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>238333</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>40298</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>343108</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:rowOff>145073</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5535,7 +5685,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3857833" y="1000125"/>
+          <a:off x="3843179" y="992798"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -5647,13 +5797,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>230050</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>334825</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5714,13 +5864,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>247652</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>41413</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>352427</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>146188</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5781,13 +5931,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>242889</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>50938</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>347664</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>155713</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5848,13 +5998,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>259948</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>364723</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -5915,13 +6065,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>240898</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>345673</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6049,13 +6199,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>255185</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>359960</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6072,73 +6222,6 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="8116973" y="1952625"/>
-          <a:ext cx="104775" cy="104775"/>
-        </a:xfrm>
-        <a:prstGeom prst="noSmoking">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="FF0000"/>
-        </a:solidFill>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="pt-BR" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>245660</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>350435</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="36" name="Símbolo de &quot;Não Permitido&quot; 35">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05756E94-8483-443D-8644-5B0E9595CBB3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8107448" y="1000125"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -6250,13 +6333,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>237377</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>342152</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6317,13 +6400,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>254979</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>41413</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>359754</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>146188</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6384,13 +6467,13 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>250216</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>50938</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>354991</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>155713</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6451,13 +6534,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>273136</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>43961</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>377911</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>148736</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6518,13 +6601,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>254086</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>358861</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6652,13 +6735,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>268373</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>373148</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6719,13 +6802,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>258848</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>363623</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6853,13 +6936,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>250565</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>53486</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>355340</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>158261</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6920,13 +7003,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>268167</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>47274</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>372942</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>152049</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6987,13 +7070,13 @@
     <xdr:from>
       <xdr:col>18</xdr:col>
       <xdr:colOff>263404</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>56799</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>368179</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>161574</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7054,13 +7137,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>257018</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>49823</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>361793</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>154598</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7121,13 +7204,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>237968</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>59348</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>342743</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>164123</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7255,13 +7338,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>252255</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>59348</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>357030</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>164123</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7322,13 +7405,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>242730</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>59348</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>347505</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>164123</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7456,13 +7539,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>234447</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>59348</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>339222</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>164123</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7523,13 +7606,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>252049</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>53136</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>356824</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>157911</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7590,13 +7673,13 @@
     <xdr:from>
       <xdr:col>25</xdr:col>
       <xdr:colOff>247286</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>62661</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>352061</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>167436</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7613,6 +7696,73 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="16622959" y="1586661"/>
+          <a:ext cx="104775" cy="104775"/>
+        </a:xfrm>
+        <a:prstGeom prst="noSmoking">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>246026</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>53486</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>350801</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>158261</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="59" name="Símbolo de &quot;Não Permitido&quot; 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05D4F59D-032A-4A6D-A623-96B98F8B3C62}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8107814" y="1005986"/>
           <a:ext cx="104775" cy="104775"/>
         </a:xfrm>
         <a:prstGeom prst="noSmoking">
@@ -7963,43 +8113,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="103" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="89"/>
-      <c r="G1" s="89"/>
-      <c r="H1" s="89"/>
-      <c r="I1" s="89"/>
-      <c r="J1" s="89"/>
-      <c r="K1" s="89"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="89"/>
-      <c r="P1" s="89"/>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="89"/>
-      <c r="S1" s="89"/>
-      <c r="T1" s="89"/>
-      <c r="U1" s="89"/>
-      <c r="V1" s="89"/>
-      <c r="W1" s="89"/>
-      <c r="X1" s="89"/>
-      <c r="Y1" s="89"/>
-      <c r="Z1" s="89"/>
-      <c r="AA1" s="89"/>
-      <c r="AB1" s="89"/>
-      <c r="AC1" s="89"/>
-      <c r="AD1" s="89"/>
-      <c r="AE1" s="89"/>
-      <c r="AF1" s="89"/>
+      <c r="B1" s="104"/>
+      <c r="C1" s="104"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="104"/>
+      <c r="K1" s="104"/>
+      <c r="L1" s="104"/>
+      <c r="M1" s="104"/>
+      <c r="N1" s="104"/>
+      <c r="O1" s="104"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="104"/>
+      <c r="R1" s="104"/>
+      <c r="S1" s="104"/>
+      <c r="T1" s="104"/>
+      <c r="U1" s="104"/>
+      <c r="V1" s="104"/>
+      <c r="W1" s="104"/>
+      <c r="X1" s="104"/>
+      <c r="Y1" s="104"/>
+      <c r="Z1" s="104"/>
+      <c r="AA1" s="104"/>
+      <c r="AB1" s="104"/>
+      <c r="AC1" s="104"/>
+      <c r="AD1" s="104"/>
+      <c r="AE1" s="104"/>
+      <c r="AF1" s="104"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="101" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="24">
@@ -8097,7 +8247,7 @@
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="87"/>
+      <c r="A3" s="102"/>
       <c r="B3" s="24" t="s">
         <v>15</v>
       </c>
@@ -8742,10 +8892,10 @@
     </row>
     <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="96" t="s">
+      <c r="A19" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="97"/>
+      <c r="B19" s="112"/>
       <c r="C19" s="29" t="s">
         <v>28</v>
       </c>
@@ -8812,11 +8962,11 @@
       <c r="K26" s="5"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="98" t="s">
+      <c r="A27" s="113" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="99"/>
-      <c r="C27" s="100"/>
+      <c r="B27" s="114"/>
+      <c r="C27" s="115"/>
       <c r="D27" s="29" t="s">
         <v>30</v>
       </c>
@@ -8847,13 +8997,13 @@
       <c r="A30" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B30" s="90" t="s">
+      <c r="B30" s="105" t="s">
         <v>26</v>
       </c>
-      <c r="C30" s="92">
+      <c r="C30" s="107">
         <v>1.03</v>
       </c>
-      <c r="D30" s="94">
+      <c r="D30" s="109">
         <v>4.12</v>
       </c>
     </row>
@@ -8861,9 +9011,9 @@
       <c r="A31" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B31" s="91"/>
-      <c r="C31" s="93"/>
-      <c r="D31" s="95"/>
+      <c r="B31" s="106"/>
+      <c r="C31" s="108"/>
+      <c r="D31" s="110"/>
       <c r="H31" s="6"/>
     </row>
   </sheetData>
@@ -8893,43 +9043,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A1" s="106" t="s">
+      <c r="A1" s="124" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
-      <c r="S1" s="107"/>
-      <c r="T1" s="107"/>
-      <c r="U1" s="107"/>
-      <c r="V1" s="107"/>
-      <c r="W1" s="107"/>
-      <c r="X1" s="107"/>
-      <c r="Y1" s="107"/>
-      <c r="Z1" s="107"/>
-      <c r="AA1" s="107"/>
-      <c r="AB1" s="107"/>
-      <c r="AC1" s="107"/>
-      <c r="AD1" s="107"/>
-      <c r="AE1" s="107"/>
-      <c r="AF1" s="107"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
+      <c r="F1" s="125"/>
+      <c r="G1" s="125"/>
+      <c r="H1" s="125"/>
+      <c r="I1" s="125"/>
+      <c r="J1" s="125"/>
+      <c r="K1" s="125"/>
+      <c r="L1" s="125"/>
+      <c r="M1" s="125"/>
+      <c r="N1" s="125"/>
+      <c r="O1" s="125"/>
+      <c r="P1" s="125"/>
+      <c r="Q1" s="125"/>
+      <c r="R1" s="125"/>
+      <c r="S1" s="125"/>
+      <c r="T1" s="125"/>
+      <c r="U1" s="125"/>
+      <c r="V1" s="125"/>
+      <c r="W1" s="125"/>
+      <c r="X1" s="125"/>
+      <c r="Y1" s="125"/>
+      <c r="Z1" s="125"/>
+      <c r="AA1" s="125"/>
+      <c r="AB1" s="125"/>
+      <c r="AC1" s="125"/>
+      <c r="AD1" s="125"/>
+      <c r="AE1" s="125"/>
+      <c r="AF1" s="125"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="126" t="s">
         <v>14</v>
       </c>
       <c r="B2" s="50">
@@ -9027,7 +9177,7 @@
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="109"/>
+      <c r="A3" s="127"/>
       <c r="B3" s="50" t="s">
         <v>18</v>
       </c>
@@ -9939,11 +10089,11 @@
       <c r="B14" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="J14" s="103" t="s">
+      <c r="J14" s="121" t="s">
         <v>44</v>
       </c>
-      <c r="K14" s="104"/>
-      <c r="L14" s="105"/>
+      <c r="K14" s="122"/>
+      <c r="L14" s="123"/>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" s="38" t="s">
@@ -9953,11 +10103,11 @@
         <f>SUM(B4:AF4)</f>
         <v>198910</v>
       </c>
-      <c r="J15" s="110" t="s">
+      <c r="J15" s="128" t="s">
         <v>45</v>
       </c>
-      <c r="K15" s="110"/>
-      <c r="L15" s="110"/>
+      <c r="K15" s="128"/>
+      <c r="L15" s="128"/>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
@@ -9967,21 +10117,21 @@
         <f>SUM(B5:AF5)</f>
         <v>4270420</v>
       </c>
-      <c r="J16" s="101" t="s">
+      <c r="J16" s="119" t="s">
         <v>46</v>
       </c>
-      <c r="K16" s="101"/>
-      <c r="L16" s="101"/>
-      <c r="R16" s="113" t="s">
+      <c r="K16" s="119"/>
+      <c r="L16" s="119"/>
+      <c r="R16" s="131" t="s">
         <v>40</v>
       </c>
-      <c r="S16" s="113"/>
-      <c r="U16" s="114" t="s">
+      <c r="S16" s="131"/>
+      <c r="U16" s="132" t="s">
         <v>55</v>
       </c>
-      <c r="V16" s="114"/>
-      <c r="W16" s="114"/>
-      <c r="X16" s="114"/>
+      <c r="V16" s="132"/>
+      <c r="W16" s="132"/>
+      <c r="X16" s="132"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
@@ -9991,23 +10141,23 @@
         <f>SUM(B6:AF6)</f>
         <v>2568430</v>
       </c>
-      <c r="J17" s="102" t="s">
+      <c r="J17" s="120" t="s">
         <v>48</v>
       </c>
-      <c r="K17" s="102"/>
-      <c r="L17" s="102"/>
-      <c r="R17" s="112" t="s">
+      <c r="K17" s="120"/>
+      <c r="L17" s="120"/>
+      <c r="R17" s="130" t="s">
         <v>54</v>
       </c>
-      <c r="S17" s="112"/>
+      <c r="S17" s="130"/>
       <c r="U17" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="V17" s="115" t="s">
+      <c r="V17" s="133" t="s">
         <v>59</v>
       </c>
-      <c r="W17" s="115"/>
-      <c r="X17" s="115"/>
+      <c r="W17" s="133"/>
+      <c r="X17" s="133"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
@@ -10017,21 +10167,21 @@
         <f>SUM(B7:AF7)</f>
         <v>2352840.9819999994</v>
       </c>
-      <c r="J18" s="101" t="s">
+      <c r="J18" s="119" t="s">
         <v>47</v>
       </c>
-      <c r="K18" s="101"/>
-      <c r="L18" s="101"/>
-      <c r="R18" s="112"/>
-      <c r="S18" s="112"/>
+      <c r="K18" s="119"/>
+      <c r="L18" s="119"/>
+      <c r="R18" s="130"/>
+      <c r="S18" s="130"/>
       <c r="U18" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="V18" s="115" t="s">
+      <c r="V18" s="133" t="s">
         <v>57</v>
       </c>
-      <c r="W18" s="115"/>
-      <c r="X18" s="115"/>
+      <c r="W18" s="133"/>
+      <c r="X18" s="133"/>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
@@ -10041,13 +10191,13 @@
         <f>SUM(B8:AF8)</f>
         <v>18000</v>
       </c>
-      <c r="J19" s="111" t="s">
+      <c r="J19" s="129" t="s">
         <v>49</v>
       </c>
-      <c r="K19" s="111"/>
-      <c r="L19" s="111"/>
-      <c r="R19" s="112"/>
-      <c r="S19" s="112"/>
+      <c r="K19" s="129"/>
+      <c r="L19" s="129"/>
+      <c r="R19" s="130"/>
+      <c r="S19" s="130"/>
       <c r="AB19" s="85"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
@@ -10058,13 +10208,13 @@
         <f t="shared" ref="B20:B21" si="8">SUM(B11:AF11)</f>
         <v>3180240</v>
       </c>
-      <c r="J20" s="101" t="s">
+      <c r="J20" s="119" t="s">
         <v>50</v>
       </c>
-      <c r="K20" s="101"/>
-      <c r="L20" s="101"/>
-      <c r="R20" s="112"/>
-      <c r="S20" s="112"/>
+      <c r="K20" s="119"/>
+      <c r="L20" s="119"/>
+      <c r="R20" s="130"/>
+      <c r="S20" s="130"/>
     </row>
     <row r="21" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
@@ -10074,22 +10224,22 @@
         <f t="shared" si="8"/>
         <v>100000</v>
       </c>
-      <c r="R21" s="112"/>
-      <c r="S21" s="112"/>
+      <c r="R21" s="130"/>
+      <c r="S21" s="130"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="R22" s="112"/>
-      <c r="S22" s="112"/>
+      <c r="R22" s="130"/>
+      <c r="S22" s="130"/>
     </row>
     <row r="23" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="R23" s="112"/>
-      <c r="S23" s="112"/>
+      <c r="R23" s="130"/>
+      <c r="S23" s="130"/>
     </row>
     <row r="24" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="96" t="s">
+      <c r="A24" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="97"/>
+      <c r="B24" s="112"/>
       <c r="C24" s="29" t="s">
         <v>28</v>
       </c>
@@ -10153,11 +10303,11 @@
     </row>
     <row r="31" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="98" t="s">
+      <c r="A32" s="113" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="99"/>
-      <c r="C32" s="100"/>
+      <c r="B32" s="114"/>
+      <c r="C32" s="115"/>
       <c r="D32" s="29" t="s">
         <v>30</v>
       </c>
@@ -10188,13 +10338,13 @@
       <c r="A35" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B35" s="90" t="s">
+      <c r="B35" s="105" t="s">
         <v>26</v>
       </c>
-      <c r="C35" s="92">
+      <c r="C35" s="107">
         <v>1.03</v>
       </c>
-      <c r="D35" s="94">
+      <c r="D35" s="109">
         <v>4.12</v>
       </c>
     </row>
@@ -10202,9 +10352,9 @@
       <c r="A36" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B36" s="91"/>
-      <c r="C36" s="93"/>
-      <c r="D36" s="95"/>
+      <c r="B36" s="106"/>
+      <c r="C36" s="108"/>
+      <c r="D36" s="110"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -10323,13 +10473,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
     <mergeCell ref="J20:L20"/>
     <mergeCell ref="J17:L17"/>
     <mergeCell ref="J14:L14"/>
@@ -10344,8 +10487,20 @@
     <mergeCell ref="U16:X16"/>
     <mergeCell ref="V17:X17"/>
     <mergeCell ref="V18:X18"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="A12:XFD12">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>$I$12</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -10354,240 +10509,241 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16DC30B1-47A1-4355-B770-E78E7C1BB711}">
-  <dimension ref="A1:AF47"/>
+  <dimension ref="A1:AF53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
     <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A1" s="106" t="s">
-        <v>32</v>
-      </c>
-      <c r="B1" s="107"/>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="107"/>
-      <c r="J1" s="107"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="107"/>
-      <c r="M1" s="107"/>
-      <c r="N1" s="107"/>
-      <c r="O1" s="107"/>
-      <c r="P1" s="107"/>
-      <c r="Q1" s="107"/>
-      <c r="R1" s="107"/>
-      <c r="S1" s="107"/>
-      <c r="T1" s="107"/>
-      <c r="U1" s="107"/>
-      <c r="V1" s="107"/>
-      <c r="W1" s="107"/>
-      <c r="X1" s="107"/>
-      <c r="Y1" s="107"/>
-      <c r="Z1" s="107"/>
-      <c r="AA1" s="107"/>
-      <c r="AB1" s="107"/>
-      <c r="AC1" s="107"/>
-      <c r="AD1" s="107"/>
-      <c r="AE1" s="107"/>
-      <c r="AF1" s="107"/>
+      <c r="A1" s="140" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="141"/>
+      <c r="C1" s="141"/>
+      <c r="D1" s="141"/>
+      <c r="E1" s="141"/>
+      <c r="F1" s="141"/>
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
+      <c r="M1" s="141"/>
+      <c r="N1" s="141"/>
+      <c r="O1" s="141"/>
+      <c r="P1" s="141"/>
+      <c r="Q1" s="141"/>
+      <c r="R1" s="141"/>
+      <c r="S1" s="141"/>
+      <c r="T1" s="141"/>
+      <c r="U1" s="141"/>
+      <c r="V1" s="141"/>
+      <c r="W1" s="141"/>
+      <c r="X1" s="141"/>
+      <c r="Y1" s="141"/>
+      <c r="Z1" s="141"/>
+      <c r="AA1" s="141"/>
+      <c r="AB1" s="141"/>
+      <c r="AC1" s="141"/>
+      <c r="AD1" s="141"/>
+      <c r="AE1" s="141"/>
+      <c r="AF1" s="141"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="142" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="50">
+      <c r="B2" s="89">
         <v>1</v>
       </c>
-      <c r="C2" s="50">
+      <c r="C2" s="89">
         <v>2</v>
       </c>
-      <c r="D2" s="50">
+      <c r="D2" s="89">
         <v>3</v>
       </c>
-      <c r="E2" s="50">
+      <c r="E2" s="89">
         <v>4</v>
       </c>
-      <c r="F2" s="50">
+      <c r="F2" s="89">
         <v>5</v>
       </c>
-      <c r="G2" s="50">
+      <c r="G2" s="89">
         <v>6</v>
       </c>
-      <c r="H2" s="50">
+      <c r="H2" s="89">
         <v>7</v>
       </c>
-      <c r="I2" s="50">
+      <c r="I2" s="89">
         <v>8</v>
       </c>
-      <c r="J2" s="50">
+      <c r="J2" s="89">
         <v>9</v>
       </c>
-      <c r="K2" s="50">
+      <c r="K2" s="89">
         <v>10</v>
       </c>
-      <c r="L2" s="50">
+      <c r="L2" s="89">
         <v>11</v>
       </c>
-      <c r="M2" s="50">
+      <c r="M2" s="89">
         <v>12</v>
       </c>
-      <c r="N2" s="50">
+      <c r="N2" s="89">
         <v>13</v>
       </c>
-      <c r="O2" s="50">
+      <c r="O2" s="89">
         <v>14</v>
       </c>
-      <c r="P2" s="51">
+      <c r="P2" s="90">
         <v>15</v>
       </c>
-      <c r="Q2" s="51">
+      <c r="Q2" s="90">
         <v>16</v>
       </c>
-      <c r="R2" s="51">
+      <c r="R2" s="90">
         <v>17</v>
       </c>
-      <c r="S2" s="51">
+      <c r="S2" s="90">
         <v>18</v>
       </c>
-      <c r="T2" s="51">
+      <c r="T2" s="90">
         <v>19</v>
       </c>
-      <c r="U2" s="51">
+      <c r="U2" s="90">
         <v>20</v>
       </c>
-      <c r="V2" s="51">
+      <c r="V2" s="90">
         <v>21</v>
       </c>
-      <c r="W2" s="51">
+      <c r="W2" s="90">
         <v>22</v>
       </c>
-      <c r="X2" s="51">
+      <c r="X2" s="90">
         <v>23</v>
       </c>
-      <c r="Y2" s="51">
+      <c r="Y2" s="90">
         <v>24</v>
       </c>
-      <c r="Z2" s="51">
+      <c r="Z2" s="90">
         <v>25</v>
       </c>
-      <c r="AA2" s="51">
+      <c r="AA2" s="90">
         <v>26</v>
       </c>
-      <c r="AB2" s="51">
+      <c r="AB2" s="90">
         <v>27</v>
       </c>
-      <c r="AC2" s="51">
+      <c r="AC2" s="90">
         <v>28</v>
       </c>
-      <c r="AD2" s="51">
+      <c r="AD2" s="90">
         <v>29</v>
       </c>
-      <c r="AE2" s="51">
+      <c r="AE2" s="90">
         <v>30</v>
       </c>
-      <c r="AF2" s="51">
+      <c r="AF2" s="90">
         <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="109"/>
-      <c r="B3" s="50" t="s">
+      <c r="A3" s="143"/>
+      <c r="B3" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="H3" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="50" t="s">
+      <c r="I3" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="50" t="s">
+      <c r="J3" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="50" t="s">
+      <c r="K3" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="50" t="s">
+      <c r="L3" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="50" t="s">
+      <c r="M3" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="50" t="s">
+      <c r="N3" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="50" t="s">
+      <c r="O3" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="50" t="s">
+      <c r="P3" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="50" t="s">
+      <c r="Q3" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="50" t="s">
+      <c r="R3" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="S3" s="50" t="s">
+      <c r="S3" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="T3" s="50" t="s">
+      <c r="T3" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="50" t="s">
+      <c r="U3" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="50" t="s">
+      <c r="V3" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="W3" s="50" t="s">
+      <c r="W3" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="X3" s="50" t="s">
+      <c r="X3" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="Y3" s="50" t="s">
+      <c r="Y3" s="89" t="s">
         <v>22</v>
       </c>
-      <c r="Z3" s="50" t="s">
+      <c r="Z3" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="AA3" s="50" t="s">
+      <c r="AA3" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="AB3" s="50" t="s">
+      <c r="AB3" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="AC3" s="50" t="s">
+      <c r="AC3" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="AD3" s="50" t="s">
+      <c r="AD3" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="AE3" s="50" t="s">
+      <c r="AE3" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="AF3" s="50" t="s">
+      <c r="AF3" s="89" t="s">
         <v>22</v>
       </c>
     </row>
@@ -10595,23 +10751,47 @@
       <c r="A4" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
+      <c r="B4" s="36">
+        <v>6490</v>
+      </c>
+      <c r="C4" s="36">
+        <v>870</v>
+      </c>
+      <c r="D4" s="36">
+        <v>1780</v>
+      </c>
       <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
+      <c r="F4" s="36">
+        <v>13910</v>
+      </c>
+      <c r="G4" s="36">
+        <v>2540</v>
+      </c>
+      <c r="H4" s="36">
+        <v>9430</v>
+      </c>
+      <c r="I4" s="36">
+        <v>4560</v>
+      </c>
+      <c r="J4" s="36">
+        <v>6900</v>
+      </c>
+      <c r="K4" s="36">
+        <v>290</v>
+      </c>
       <c r="L4" s="46"/>
-      <c r="M4" s="121" t="s">
+      <c r="M4" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="1"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
+      <c r="N4" s="1">
+        <v>16990</v>
+      </c>
+      <c r="O4" s="36">
+        <v>4530</v>
+      </c>
+      <c r="P4" s="36">
+        <v>3920</v>
+      </c>
       <c r="Q4" s="36"/>
       <c r="R4" s="46"/>
       <c r="S4" s="46"/>
@@ -10633,25 +10813,49 @@
       <c r="A5" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="36"/>
+      <c r="B5" s="36">
+        <v>159990</v>
+      </c>
+      <c r="C5" s="8">
+        <v>139910</v>
+      </c>
+      <c r="D5" s="36">
+        <v>111310</v>
+      </c>
       <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="36"/>
-      <c r="K5" s="36"/>
+      <c r="F5" s="36">
+        <v>154730</v>
+      </c>
+      <c r="G5" s="36">
+        <v>111710</v>
+      </c>
+      <c r="H5" s="36">
+        <v>171350</v>
+      </c>
+      <c r="I5" s="36">
+        <v>195630</v>
+      </c>
+      <c r="J5" s="36">
+        <v>197840</v>
+      </c>
+      <c r="K5" s="36">
+        <v>110520</v>
+      </c>
       <c r="L5" s="36"/>
-      <c r="M5" s="121" t="s">
+      <c r="M5" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="N5" s="8"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
+      <c r="N5" s="8">
+        <v>236030</v>
+      </c>
+      <c r="O5" s="36">
+        <v>168120</v>
+      </c>
+      <c r="P5" s="36">
+        <v>111520</v>
+      </c>
       <c r="Q5" s="36"/>
-      <c r="R5" s="40"/>
+      <c r="R5" s="36"/>
       <c r="S5" s="36"/>
       <c r="T5" s="36"/>
       <c r="U5" s="36"/>
@@ -10661,7 +10865,7 @@
       <c r="Y5" s="36"/>
       <c r="Z5" s="36"/>
       <c r="AA5" s="36"/>
-      <c r="AB5" s="40"/>
+      <c r="AB5" s="36"/>
       <c r="AC5" s="36"/>
       <c r="AD5" s="36"/>
       <c r="AE5" s="36"/>
@@ -10671,23 +10875,47 @@
       <c r="A6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="36"/>
+      <c r="B6" s="36">
+        <v>5580</v>
+      </c>
+      <c r="C6" s="8">
+        <v>6650</v>
+      </c>
+      <c r="D6" s="36">
+        <v>5780</v>
+      </c>
       <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="36"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="36"/>
+      <c r="F6" s="36">
+        <v>6310</v>
+      </c>
+      <c r="G6" s="36">
+        <v>5280</v>
+      </c>
+      <c r="H6" s="36">
+        <v>6290</v>
+      </c>
+      <c r="I6" s="36">
+        <v>5460</v>
+      </c>
+      <c r="J6" s="36">
+        <v>9820</v>
+      </c>
+      <c r="K6" s="36">
+        <v>2570</v>
+      </c>
       <c r="L6" s="36"/>
-      <c r="M6" s="121" t="s">
+      <c r="M6" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="N6" s="8"/>
-      <c r="O6" s="36"/>
-      <c r="P6" s="119"/>
+      <c r="N6" s="8">
+        <v>8580</v>
+      </c>
+      <c r="O6" s="36">
+        <v>6350</v>
+      </c>
+      <c r="P6" s="86">
+        <v>4550</v>
+      </c>
       <c r="Q6" s="36"/>
       <c r="R6" s="36"/>
       <c r="S6" s="36"/>
@@ -10706,26 +10934,54 @@
       <c r="AF6" s="36"/>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A7" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="36"/>
-      <c r="K7" s="36"/>
-      <c r="L7" s="36"/>
-      <c r="M7" s="121" t="s">
-        <v>23</v>
-      </c>
-      <c r="N7" s="36"/>
-      <c r="O7" s="36"/>
-      <c r="P7" s="119"/>
+      <c r="A7" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="36">
+        <v>90850</v>
+      </c>
+      <c r="C7" s="8">
+        <v>95430</v>
+      </c>
+      <c r="D7" s="36">
+        <v>111310</v>
+      </c>
+      <c r="E7" s="36">
+        <v>6360</v>
+      </c>
+      <c r="F7" s="36">
+        <v>86820</v>
+      </c>
+      <c r="G7" s="36">
+        <v>142920</v>
+      </c>
+      <c r="H7" s="36">
+        <v>94950</v>
+      </c>
+      <c r="I7" s="36">
+        <v>94950</v>
+      </c>
+      <c r="J7" s="36">
+        <v>95190</v>
+      </c>
+      <c r="K7" s="36">
+        <v>108510</v>
+      </c>
+      <c r="L7" s="36">
+        <v>14450</v>
+      </c>
+      <c r="M7" s="8">
+        <v>77440</v>
+      </c>
+      <c r="N7" s="8">
+        <v>104180</v>
+      </c>
+      <c r="O7" s="36">
+        <v>99020</v>
+      </c>
+      <c r="P7" s="86">
+        <v>42550</v>
+      </c>
       <c r="Q7" s="36"/>
       <c r="R7" s="36"/>
       <c r="S7" s="36"/>
@@ -10745,30 +11001,66 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="48" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="47"/>
-      <c r="E8" s="47"/>
-      <c r="F8" s="47"/>
-      <c r="G8" s="47"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="47"/>
-      <c r="J8" s="36"/>
-      <c r="K8" s="47"/>
-      <c r="L8" s="47"/>
-      <c r="M8" s="121" t="s">
-        <v>23</v>
-      </c>
-      <c r="N8" s="8"/>
-      <c r="O8" s="36"/>
-      <c r="P8" s="119"/>
+        <v>40</v>
+      </c>
+      <c r="B8" s="36">
+        <f>(B7*(1-$B$48))+B6</f>
+        <v>92568.875</v>
+      </c>
+      <c r="C8" s="36">
+        <f t="shared" ref="C8:D8" si="0">(C7*(1-$B$48))+C6</f>
+        <v>98024.225000000006</v>
+      </c>
+      <c r="D8" s="36">
+        <f t="shared" si="0"/>
+        <v>112359.325</v>
+      </c>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36">
+        <f t="shared" ref="F8" si="1">(F7*(1-$B$48))+F6</f>
+        <v>89440.150000000009</v>
+      </c>
+      <c r="G8" s="36">
+        <f t="shared" ref="G8" si="2">(G7*(1-$B$48))+G6</f>
+        <v>142125.9</v>
+      </c>
+      <c r="H8" s="36">
+        <f t="shared" ref="H8" si="3">(H7*(1-$B$48))+H6</f>
+        <v>97204.625</v>
+      </c>
+      <c r="I8" s="36">
+        <f t="shared" ref="I8" si="4">(I7*(1-$B$48))+I6</f>
+        <v>96374.625</v>
+      </c>
+      <c r="J8" s="36">
+        <f t="shared" ref="J8" si="5">(J7*(1-$B$48))+J6</f>
+        <v>100964.425</v>
+      </c>
+      <c r="K8" s="36">
+        <f t="shared" ref="K8" si="6">(K7*(1-$B$48))+K6</f>
+        <v>106468.325</v>
+      </c>
+      <c r="L8" s="36"/>
+      <c r="M8" s="8">
+        <v>77440</v>
+      </c>
+      <c r="N8" s="36">
+        <f t="shared" ref="N8" si="7">(N7*(1-$B$48))+N6</f>
+        <v>108332.35</v>
+      </c>
+      <c r="O8" s="36">
+        <f t="shared" ref="O8" si="8">(O7*(1-$B$48))+O6</f>
+        <v>101161.65000000001</v>
+      </c>
+      <c r="P8" s="36">
+        <f t="shared" ref="P8" si="9">(P7*(1-$B$48))+P6</f>
+        <v>45291.625</v>
+      </c>
       <c r="Q8" s="36"/>
       <c r="R8" s="36"/>
       <c r="S8" s="36"/>
       <c r="T8" s="36"/>
-      <c r="U8" s="26"/>
+      <c r="U8" s="36"/>
       <c r="V8" s="36"/>
       <c r="W8" s="36"/>
       <c r="X8" s="36"/>
@@ -10782,26 +11074,50 @@
       <c r="AF8" s="36"/>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A9" s="84" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="47"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="47"/>
+      <c r="A9" s="48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="47">
+        <v>410</v>
+      </c>
+      <c r="C9" s="8">
+        <v>590</v>
+      </c>
+      <c r="D9" s="47">
+        <v>1100</v>
+      </c>
       <c r="E9" s="47"/>
-      <c r="F9" s="47"/>
-      <c r="G9" s="47"/>
-      <c r="H9" s="120"/>
-      <c r="I9" s="47"/>
-      <c r="J9" s="47"/>
-      <c r="K9" s="36"/>
+      <c r="F9" s="47">
+        <v>1080</v>
+      </c>
+      <c r="G9" s="47">
+        <v>880</v>
+      </c>
+      <c r="H9" s="47">
+        <v>940</v>
+      </c>
+      <c r="I9" s="47">
+        <v>980</v>
+      </c>
+      <c r="J9" s="36">
+        <v>1330</v>
+      </c>
+      <c r="K9" s="47">
+        <v>1140</v>
+      </c>
       <c r="L9" s="47"/>
-      <c r="M9" s="121" t="s">
-        <v>23</v>
-      </c>
-      <c r="N9" s="8"/>
-      <c r="O9" s="36"/>
-      <c r="P9" s="36"/>
+      <c r="M9" s="8">
+        <v>1170</v>
+      </c>
+      <c r="N9" s="8">
+        <v>990</v>
+      </c>
+      <c r="O9" s="36">
+        <v>0</v>
+      </c>
+      <c r="P9" s="86">
+        <v>1070</v>
+      </c>
       <c r="Q9" s="36"/>
       <c r="R9" s="36"/>
       <c r="S9" s="36"/>
@@ -10820,102 +11136,177 @@
       <c r="AF9" s="36"/>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A10" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
+      <c r="A10" s="84" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="47">
+        <v>40210</v>
+      </c>
+      <c r="C10" s="8">
+        <v>42100</v>
+      </c>
       <c r="D10" s="47"/>
       <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="46"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-      <c r="K10" s="47"/>
+      <c r="F10" s="47">
+        <v>42660</v>
+      </c>
+      <c r="G10" s="47">
+        <v>48070</v>
+      </c>
+      <c r="H10" s="40">
+        <v>39990</v>
+      </c>
+      <c r="I10" s="47">
+        <v>45970</v>
+      </c>
+      <c r="J10" s="47">
+        <v>43970</v>
+      </c>
+      <c r="K10" s="36"/>
       <c r="L10" s="47"/>
-      <c r="M10" s="121" t="s">
+      <c r="M10" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="N10" s="8"/>
-      <c r="O10" s="47"/>
-      <c r="P10" s="47"/>
-      <c r="Q10" s="47"/>
-      <c r="R10" s="47"/>
-      <c r="S10" s="47"/>
-      <c r="T10" s="47"/>
-      <c r="U10" s="47"/>
-      <c r="V10" s="47"/>
-      <c r="W10" s="47"/>
-      <c r="X10" s="47"/>
-      <c r="Y10" s="47"/>
-      <c r="Z10" s="47"/>
-      <c r="AA10" s="47"/>
-      <c r="AB10" s="47"/>
-      <c r="AC10" s="47"/>
-      <c r="AD10" s="47"/>
-      <c r="AE10" s="47"/>
+      <c r="N10" s="8">
+        <v>39300</v>
+      </c>
+      <c r="O10" s="36">
+        <v>40330</v>
+      </c>
+      <c r="P10" s="36">
+        <v>40300</v>
+      </c>
+      <c r="Q10" s="36"/>
+      <c r="R10" s="36"/>
+      <c r="S10" s="36"/>
+      <c r="T10" s="36"/>
+      <c r="U10" s="26"/>
+      <c r="V10" s="36"/>
+      <c r="W10" s="36"/>
+      <c r="X10" s="36"/>
+      <c r="Y10" s="36"/>
+      <c r="Z10" s="36"/>
+      <c r="AA10" s="36"/>
+      <c r="AB10" s="36"/>
+      <c r="AC10" s="36"/>
+      <c r="AD10" s="36"/>
+      <c r="AE10" s="36"/>
       <c r="AF10" s="36"/>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="36"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="36"/>
-      <c r="J11" s="36"/>
-      <c r="K11" s="36"/>
-      <c r="L11" s="36"/>
-      <c r="M11" s="121" t="s">
+      <c r="A11" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="47">
+        <f>B10*(1-$B$48)</f>
+        <v>38501.074999999997</v>
+      </c>
+      <c r="C11" s="47">
+        <f t="shared" ref="C11" si="10">C10*(1-$B$48)</f>
+        <v>40310.75</v>
+      </c>
+      <c r="D11" s="47">
+        <v>36570</v>
+      </c>
+      <c r="E11" s="47"/>
+      <c r="F11" s="47">
+        <f t="shared" ref="F11" si="11">F10*(1-$B$48)</f>
+        <v>40846.950000000004</v>
+      </c>
+      <c r="G11" s="47">
+        <f t="shared" ref="G11" si="12">G10*(1-$B$48)</f>
+        <v>46027.025000000001</v>
+      </c>
+      <c r="H11" s="47">
+        <f t="shared" ref="H11" si="13">H10*(1-$B$48)</f>
+        <v>38290.425000000003</v>
+      </c>
+      <c r="I11" s="47">
+        <f t="shared" ref="I11" si="14">I10*(1-$B$48)</f>
+        <v>44016.275000000001</v>
+      </c>
+      <c r="J11" s="47">
+        <f t="shared" ref="J11" si="15">J10*(1-$B$48)</f>
+        <v>42101.275000000001</v>
+      </c>
+      <c r="K11" s="36">
+        <v>36860</v>
+      </c>
+      <c r="L11" s="47"/>
+      <c r="M11" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="N11" s="8"/>
-      <c r="O11" s="36"/>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="36"/>
-      <c r="R11" s="36"/>
-      <c r="S11" s="36"/>
-      <c r="T11" s="36"/>
-      <c r="U11" s="36"/>
-      <c r="V11" s="36"/>
-      <c r="W11" s="36"/>
-      <c r="X11" s="36"/>
-      <c r="Y11" s="36"/>
-      <c r="Z11" s="36"/>
-      <c r="AA11" s="36"/>
-      <c r="AB11" s="36"/>
-      <c r="AC11" s="36"/>
-      <c r="AD11" s="36"/>
-      <c r="AE11" s="36"/>
+      <c r="N11" s="47">
+        <f t="shared" ref="N11" si="16">N10*(1-$B$48)</f>
+        <v>37629.75</v>
+      </c>
+      <c r="O11" s="47">
+        <f t="shared" ref="O11" si="17">O10*(1-$B$48)</f>
+        <v>38615.974999999999</v>
+      </c>
+      <c r="P11" s="47">
+        <f t="shared" ref="P11" si="18">P10*(1-$B$48)</f>
+        <v>38587.25</v>
+      </c>
+      <c r="Q11" s="47"/>
+      <c r="R11" s="47"/>
+      <c r="S11" s="47"/>
+      <c r="T11" s="47"/>
+      <c r="U11" s="47"/>
+      <c r="V11" s="47"/>
+      <c r="W11" s="47"/>
+      <c r="X11" s="47"/>
+      <c r="Y11" s="47"/>
+      <c r="Z11" s="47"/>
+      <c r="AA11" s="47"/>
+      <c r="AB11" s="47"/>
+      <c r="AC11" s="47"/>
+      <c r="AD11" s="47"/>
+      <c r="AE11" s="47"/>
       <c r="AF11" s="36"/>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A12" s="73" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="36"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="1"/>
+      <c r="A12" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="36">
+        <v>403200</v>
+      </c>
+      <c r="C12" s="8">
+        <v>403200</v>
+      </c>
+      <c r="D12" s="36"/>
       <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="36">
+        <v>100800</v>
+      </c>
+      <c r="H12" s="87">
+        <v>0</v>
+      </c>
+      <c r="I12" s="36">
+        <v>126000</v>
+      </c>
+      <c r="J12" s="36">
+        <v>12600</v>
+      </c>
       <c r="K12" s="36"/>
       <c r="L12" s="36"/>
-      <c r="M12" s="121" t="s">
+      <c r="M12" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="N12" s="8"/>
-      <c r="O12" s="36"/>
-      <c r="P12" s="36"/>
+      <c r="N12" s="8">
+        <f>50400*7</f>
+        <v>352800</v>
+      </c>
+      <c r="O12" s="8">
+        <f>50400*6</f>
+        <v>302400</v>
+      </c>
+      <c r="P12" s="8">
+        <f>50400*6</f>
+        <v>302400</v>
+      </c>
       <c r="Q12" s="36"/>
       <c r="R12" s="36"/>
       <c r="S12" s="36"/>
@@ -10933,448 +11324,546 @@
       <c r="AE12" s="36"/>
       <c r="AF12" s="36"/>
     </row>
-    <row r="13" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="59"/>
-      <c r="B13" s="60"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="62"/>
-      <c r="F13" s="62"/>
-      <c r="G13" s="62"/>
-      <c r="H13" s="62"/>
-      <c r="I13" s="62"/>
-      <c r="J13" s="61"/>
-      <c r="K13" s="61"/>
-      <c r="L13" s="61"/>
-      <c r="M13" s="61"/>
-      <c r="N13" s="61"/>
-      <c r="O13" s="72"/>
-      <c r="P13" s="72"/>
-      <c r="Q13" s="72"/>
-      <c r="R13" s="62"/>
-      <c r="T13" s="62"/>
-      <c r="U13" s="62"/>
-      <c r="V13" s="62"/>
-      <c r="X13" s="61"/>
-      <c r="Y13" s="62"/>
-      <c r="Z13" s="62"/>
-      <c r="AA13" s="62"/>
-      <c r="AB13" s="62"/>
-      <c r="AC13" s="62"/>
-      <c r="AD13" s="62"/>
-      <c r="AE13" s="61"/>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A13" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="36">
+        <v>20000</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="H13" s="36">
+        <v>10000</v>
+      </c>
+      <c r="I13" s="36"/>
+      <c r="J13" s="36"/>
+      <c r="K13" s="36"/>
+      <c r="L13" s="36"/>
+      <c r="M13" s="88" t="s">
+        <v>23</v>
+      </c>
+      <c r="N13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="O13" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="P13" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q13" s="36" t="s">
+        <v>51</v>
+      </c>
+      <c r="R13" s="36"/>
+      <c r="S13" s="36"/>
+      <c r="T13" s="36"/>
+      <c r="U13" s="36"/>
+      <c r="V13" s="36"/>
+      <c r="W13" s="36"/>
+      <c r="X13" s="36"/>
+      <c r="Y13" s="36"/>
+      <c r="Z13" s="36"/>
+      <c r="AA13" s="36"/>
+      <c r="AB13" s="36"/>
+      <c r="AC13" s="36"/>
+      <c r="AD13" s="36"/>
+      <c r="AE13" s="36"/>
+      <c r="AF13" s="36"/>
     </row>
     <row r="14" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="17"/>
-      <c r="B14" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="J14" s="103" t="s">
-        <v>44</v>
-      </c>
-      <c r="K14" s="104"/>
-      <c r="L14" s="105"/>
+      <c r="A14" s="59"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="62"/>
+      <c r="F14" s="62"/>
+      <c r="G14" s="100"/>
+      <c r="I14" s="62"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="61"/>
+      <c r="L14" s="61"/>
+      <c r="M14" s="61"/>
+      <c r="N14" s="61"/>
+      <c r="O14" s="72"/>
+      <c r="P14" s="72"/>
+      <c r="Q14" s="72"/>
+      <c r="R14" s="62"/>
+      <c r="T14" s="62"/>
+      <c r="U14" s="62"/>
+      <c r="V14" s="62"/>
+      <c r="X14" s="61"/>
+      <c r="Y14" s="62"/>
+      <c r="Z14" s="62"/>
+      <c r="AA14" s="62"/>
+      <c r="AB14" s="62"/>
+      <c r="AC14" s="62"/>
+      <c r="AD14" s="62"/>
+      <c r="AE14" s="61"/>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A15" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="12">
-        <f>SUM(B4:AF4)</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="110" t="s">
-        <v>45</v>
-      </c>
-      <c r="K15" s="110"/>
-      <c r="L15" s="110"/>
+      <c r="A15" s="17"/>
+      <c r="B15" s="18" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="12">
+        <f t="shared" ref="B16:B21" si="19">SUM(B4:AF4)</f>
+        <v>72210</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="12">
-        <f>SUM(B5:AF5)</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="101" t="s">
-        <v>46</v>
-      </c>
-      <c r="K16" s="101"/>
-      <c r="L16" s="101"/>
-      <c r="R16" s="113" t="s">
+      <c r="B17" s="12">
+        <f t="shared" si="19"/>
+        <v>1868660</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="12">
+        <f t="shared" si="19"/>
+        <v>73220</v>
+      </c>
+      <c r="F18" s="121" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="122"/>
+      <c r="H18" s="123"/>
+      <c r="K18" s="131" t="s">
         <v>40</v>
       </c>
-      <c r="S16" s="113"/>
-      <c r="U16" s="114" t="s">
+      <c r="L18" s="131"/>
+      <c r="O18" s="132" t="s">
         <v>55</v>
       </c>
-      <c r="V16" s="114"/>
-      <c r="W16" s="114"/>
-      <c r="X16" s="114"/>
+      <c r="P18" s="132"/>
+      <c r="Q18" s="132"/>
+      <c r="R18" s="132"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="12">
-        <f>SUM(B6:AF6)</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="102" t="s">
-        <v>48</v>
-      </c>
-      <c r="K17" s="102"/>
-      <c r="L17" s="102"/>
-      <c r="R17" s="112" t="s">
-        <v>54</v>
-      </c>
-      <c r="S17" s="112"/>
-      <c r="U17" s="1" t="s">
+    <row r="19" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="12">
+        <f t="shared" si="19"/>
+        <v>1264930</v>
+      </c>
+      <c r="F19" s="144" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="145"/>
+      <c r="H19" s="146"/>
+      <c r="K19" s="130" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" s="130"/>
+      <c r="O19" s="133" t="s">
+        <v>59</v>
+      </c>
+      <c r="P19" s="133"/>
+      <c r="Q19" s="133"/>
+      <c r="R19" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="V17" s="115" t="s">
-        <v>59</v>
-      </c>
-      <c r="W17" s="115"/>
-      <c r="X17" s="115"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" s="12">
-        <f>SUM(B7:AF7)</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="101" t="s">
-        <v>47</v>
-      </c>
-      <c r="K18" s="101"/>
-      <c r="L18" s="101"/>
-      <c r="R18" s="112"/>
-      <c r="S18" s="112"/>
-      <c r="U18" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="V18" s="115" t="s">
-        <v>57</v>
-      </c>
-      <c r="W18" s="115"/>
-      <c r="X18" s="115"/>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="B19" s="12">
-        <f>SUM(B8:AF8)</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="111" t="s">
-        <v>49</v>
-      </c>
-      <c r="K19" s="111"/>
-      <c r="L19" s="111"/>
-      <c r="R19" s="112"/>
-      <c r="S19" s="112"/>
-      <c r="AB19" s="85"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
-        <v>3</v>
+      <c r="A20" s="7" t="s">
+        <v>40</v>
       </c>
       <c r="B20" s="12">
-        <f t="shared" ref="B20:B21" si="0">SUM(B11:AF11)</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="101" t="s">
-        <v>50</v>
-      </c>
-      <c r="K20" s="101"/>
-      <c r="L20" s="101"/>
-      <c r="R20" s="112"/>
-      <c r="S20" s="112"/>
+        <f t="shared" si="19"/>
+        <v>1267756.0999999999</v>
+      </c>
+      <c r="F20" s="137" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" s="138"/>
+      <c r="H20" s="139"/>
+      <c r="K20" s="130"/>
+      <c r="L20" s="130"/>
+      <c r="O20" s="133" t="s">
+        <v>57</v>
+      </c>
+      <c r="P20" s="133"/>
+      <c r="Q20" s="133"/>
+      <c r="R20" s="1" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="21" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R21" s="112"/>
-      <c r="S21" s="112"/>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" s="12">
+        <f t="shared" si="19"/>
+        <v>11680</v>
+      </c>
+      <c r="F21" s="134" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="135"/>
+      <c r="H21" s="136"/>
+      <c r="K21" s="130"/>
+      <c r="L21" s="130"/>
+      <c r="AB21" s="85"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="R22" s="112"/>
-      <c r="S22" s="112"/>
+      <c r="A22" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="12">
+        <f t="shared" ref="B22:B23" si="20">SUM(B12:AF12)</f>
+        <v>2003400</v>
+      </c>
+      <c r="F22" s="137" t="s">
+        <v>47</v>
+      </c>
+      <c r="G22" s="138"/>
+      <c r="H22" s="139"/>
+      <c r="K22" s="130"/>
+      <c r="L22" s="130"/>
     </row>
     <row r="23" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="R23" s="112"/>
-      <c r="S23" s="112"/>
+      <c r="A23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B23" s="16">
+        <f t="shared" si="20"/>
+        <v>30000</v>
+      </c>
+      <c r="F23" s="134" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" s="135"/>
+      <c r="H23" s="136"/>
+      <c r="K23" s="130"/>
+      <c r="L23" s="130"/>
     </row>
-    <row r="24" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="96" t="s">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="F24" s="137" t="s">
+        <v>50</v>
+      </c>
+      <c r="G24" s="138"/>
+      <c r="H24" s="139"/>
+      <c r="K24" s="130"/>
+      <c r="L24" s="130"/>
+    </row>
+    <row r="25" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K25" s="130"/>
+      <c r="L25" s="130"/>
+    </row>
+    <row r="26" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="97"/>
-      <c r="C24" s="29" t="s">
+      <c r="B26" s="112"/>
+      <c r="C26" s="29" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" s="11">
-        <v>100800</v>
-      </c>
-      <c r="C25" s="11">
-        <f>B25/B27</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" s="12">
-        <v>50400</v>
-      </c>
-      <c r="C26" s="12">
-        <f>B26/B27</f>
-        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="A27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="11">
+        <v>100800</v>
+      </c>
+      <c r="C27" s="11">
+        <f>B27/B29</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" s="12">
+        <v>50400</v>
+      </c>
+      <c r="C28" s="12">
+        <f>B28/B29</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="12">
+      <c r="B29" s="12">
         <v>12600</v>
       </c>
-      <c r="C27" s="12">
+      <c r="C29" s="12">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+    <row r="30" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="13">
+      <c r="B30" s="13">
         <v>10000</v>
       </c>
-      <c r="C28" s="13">
+      <c r="C30" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="31" t="s">
+    <row r="31" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="32">
+      <c r="B31" s="32">
         <v>6000</v>
       </c>
-      <c r="C29" s="13">
+      <c r="C31" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="98" t="s">
+    <row r="33" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="113" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="99"/>
-      <c r="C32" s="100"/>
-      <c r="D32" s="29" t="s">
+      <c r="B34" s="114"/>
+      <c r="C34" s="115"/>
+      <c r="D34" s="29" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B33" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="20">
-        <v>7.2050000000000001</v>
-      </c>
-      <c r="D33" s="34"/>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="22"/>
-      <c r="B34" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="C34" s="28">
-        <v>6.46</v>
-      </c>
-      <c r="D34" s="35"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B35" s="90" t="s">
-        <v>26</v>
-      </c>
-      <c r="C35" s="92">
-        <v>1.03</v>
-      </c>
-      <c r="D35" s="94">
-        <v>4.12</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="20">
+        <v>7.2050000000000001</v>
+      </c>
+      <c r="D35" s="34"/>
     </row>
     <row r="36" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="22"/>
+      <c r="B36" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="28">
+        <v>6.46</v>
+      </c>
+      <c r="D36" s="35"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B37" s="105" t="s">
+        <v>26</v>
+      </c>
+      <c r="C37" s="107">
+        <v>1.03</v>
+      </c>
+      <c r="D37" s="109">
+        <v>4.12</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B36" s="91"/>
-      <c r="C36" s="93"/>
-      <c r="D36" s="95"/>
+      <c r="B38" s="106"/>
+      <c r="C38" s="108"/>
+      <c r="D38" s="110"/>
     </row>
-    <row r="38" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="116" t="s">
+    <row r="40" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="116" t="s">
         <v>39</v>
       </c>
-      <c r="B39" s="117"/>
-      <c r="C39" s="117"/>
-      <c r="D39" s="117"/>
-      <c r="E39" s="118"/>
+      <c r="B41" s="117"/>
+      <c r="C41" s="117"/>
+      <c r="D41" s="117"/>
+      <c r="E41" s="118"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="56"/>
-      <c r="B40" s="52" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="56"/>
+      <c r="B42" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="C40" s="52" t="s">
+      <c r="C42" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="52" t="s">
+      <c r="D42" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="E40" s="53" t="s">
+      <c r="E42" s="53" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="22"/>
-      <c r="B41" s="67">
+    <row r="43" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="22"/>
+      <c r="B43" s="67">
         <v>3690</v>
       </c>
-      <c r="C41" s="67">
+      <c r="C43" s="67">
         <f>26430+1580</f>
         <v>28010</v>
       </c>
-      <c r="D41" s="67"/>
-      <c r="E41" s="68"/>
+      <c r="D43" s="67"/>
+      <c r="E43" s="68"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="64"/>
-      <c r="B42" s="65"/>
-      <c r="C42" s="65"/>
-      <c r="D42" s="65"/>
-      <c r="E42" s="66"/>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="64"/>
+      <c r="B44" s="65"/>
+      <c r="C44" s="65"/>
+      <c r="D44" s="65"/>
+      <c r="E44" s="65"/>
+      <c r="F44" s="99"/>
     </row>
-    <row r="43" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="64"/>
-      <c r="B43" s="65"/>
-      <c r="C43" s="65"/>
-      <c r="D43" s="65"/>
-      <c r="E43" s="66"/>
+    <row r="45" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="64"/>
+      <c r="B45" s="65"/>
+      <c r="C45" s="65"/>
+      <c r="D45" s="65"/>
+      <c r="E45" s="65"/>
+      <c r="F45" s="99"/>
     </row>
-    <row r="44" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="116" t="s">
+    <row r="46" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="147" t="s">
         <v>33</v>
       </c>
-      <c r="B44" s="117"/>
-      <c r="C44" s="117"/>
-      <c r="D44" s="117"/>
-      <c r="E44" s="117"/>
-      <c r="F44" s="118"/>
+      <c r="B46" s="148"/>
+      <c r="C46" s="148"/>
+      <c r="D46" s="148"/>
+      <c r="E46" s="148"/>
+      <c r="F46" s="149"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="56"/>
-      <c r="B45" s="52" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="56"/>
+      <c r="B47" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="C45" s="52" t="s">
+      <c r="C47" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="D45" s="52" t="s">
+      <c r="D47" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="E45" s="52" t="s">
+      <c r="E47" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="F45" s="79" t="s">
+      <c r="F47" s="79" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="54" t="s">
+    <row r="48" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="B46" s="57">
-        <v>0.11</v>
-      </c>
-      <c r="C46" s="57">
-        <v>0.11</v>
-      </c>
-      <c r="D46" s="70">
-        <v>0.24</v>
-      </c>
-      <c r="E46" s="57">
-        <v>4.5999999999999999E-3</v>
-      </c>
-      <c r="F46" s="80"/>
+      <c r="B48" s="97">
+        <v>4.2500000000000003E-2</v>
+      </c>
+      <c r="C48" s="97"/>
+      <c r="D48" s="95"/>
+      <c r="E48" s="95"/>
+      <c r="F48" s="80"/>
     </row>
-    <row r="47" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="55" t="s">
+    <row r="49" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="91" t="s">
         <v>41</v>
       </c>
-      <c r="B47" s="58">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="C47" s="58">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="D47" s="71">
-        <v>0.29299999999999998</v>
-      </c>
-      <c r="E47" s="58">
-        <v>3.4099999999999998E-2</v>
-      </c>
-      <c r="F47" s="81"/>
+      <c r="B49" s="98">
+        <v>5.7700000000000001E-2</v>
+      </c>
+      <c r="C49" s="98"/>
+      <c r="D49" s="96"/>
+      <c r="E49" s="96"/>
+      <c r="F49" s="81"/>
+    </row>
+    <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="116" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51" s="117"/>
+      <c r="C51" s="117"/>
+      <c r="D51" s="117"/>
+      <c r="E51" s="118"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="56"/>
+      <c r="B52" s="52" t="s">
+        <v>34</v>
+      </c>
+      <c r="C52" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" s="52" t="s">
+        <v>36</v>
+      </c>
+      <c r="E52" s="53" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="22"/>
+      <c r="B53" s="92">
+        <v>6.74</v>
+      </c>
+      <c r="C53" s="92">
+        <v>6.74</v>
+      </c>
+      <c r="D53" s="92">
+        <v>6.84</v>
+      </c>
+      <c r="E53" s="93"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="K19:L25"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="U16:X16"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="R17:S23"/>
-    <mergeCell ref="V17:X17"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="V18:X18"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="O18:R18"/>
+    <mergeCell ref="O19:Q19"/>
+    <mergeCell ref="O20:Q20"/>
+    <mergeCell ref="A46:F46"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:C38"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="A13:XFD13">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>$C$13</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>